<commit_message>
E2E checkout and update profile
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/DataCMS.xlsx
+++ b/src/test/resources/testdata/DataCMS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\ProjectAutomation\Anhtester_CMS_AutomationTestingSeleniumJavaProject\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217345EB-4BE1-4D6B-A598-43F9BA3F84E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A383B902-EBC2-4AF6-8789-B6BC4E635BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="31">
   <si>
     <t>Email</t>
   </si>
@@ -100,6 +100,27 @@
   </si>
   <si>
     <t>Dell</t>
+  </si>
+  <si>
+    <t>Screnario</t>
+  </si>
+  <si>
+    <t>Coca cola</t>
+  </si>
+  <si>
+    <t>nước giải khác</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>E2E Checkout</t>
+  </si>
+  <si>
+    <t>AddressIndex</t>
+  </si>
+  <si>
+    <t>OrderNote</t>
   </si>
 </sst>
 </file>
@@ -109,7 +130,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +163,11 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -207,7 +233,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -218,6 +244,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -609,107 +647,72 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35773BB2-78C5-472F-920D-64B227F15414}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" style="6" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="31.42578125" style="6" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="6"/>
+    <col min="1" max="1" width="16.7109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" style="13" customWidth="1"/>
+    <col min="3" max="4" width="23.5703125" style="13" customWidth="1"/>
+    <col min="5" max="8" width="31.42578125" style="13" customWidth="1"/>
+    <col min="9" max="9" width="26.42578125" style="13" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
+      <c r="F1" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="11">
+        <v>99999999999</v>
+      </c>
+      <c r="D2" s="12">
+        <v>2</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="10">
+        <v>1</v>
+      </c>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>